<commit_message>
Pass the keyword list, generic words and round multiple through the run
run_python_tests takes keywords, generic_words and round_multiple; write_working_paper takes
the same lists, so the Lines columns can't disagree with the flags, and states them on the
cover itself. make_fixtures passes the run's values to both.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample_priority_list.xlsx
+++ b/docs/sample_priority_list.xlsx
@@ -576,72 +576,72 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parameter: Large amount</t>
+          <t>Parameter: Keywords</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10 times the median non-zero amount, used in "why selected" only when performance materiality isn't set (practical judgement)</t>
+          <t>adjust, write off, reversal, correction, director, related party, cash advance, settlement, no invoice, suspense</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Parameter: Period-end windows</t>
+          <t>Parameter: Generic narration words</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>last 3 and first 2 days of each quarter; 5 working days either side of the year-end</t>
+          <t>adj, adjustment, adjusting, jv, je, journal, entry, correction, reclass, misc, miscellaneous, other, general, various, sundry, test, tbd, being</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Parameter: Weekend, holiday and round-amount tests</t>
+          <t>Parameter: Large amount</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>manual lines only</t>
+          <t>10 times the median non-zero amount, used in "why selected" only when performance materiality isn't set (practical judgement)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Parameter: Round amount</t>
+          <t>Parameter: Period-end windows</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>multiple of 10,000</t>
+          <t>last 3 and first 2 days of each quarter; 5 working days either side of the year-end</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Parameter: Keywords</t>
+          <t>Parameter: Weekend, holiday and round-amount tests</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>adjust, write off, reversal, correction, director, related party, cash advance, settlement, no invoice, suspense</t>
+          <t>manual lines only</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Parameter: Generic narration words</t>
+          <t>Parameter: Round amount</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>adj, adjustment, adjusting, jv, je, journal, entry, correction, reclass, misc, miscellaneous, other, general, various, sundry, test, tbd, being</t>
+          <t>multiple of 10,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.5.0: RunSettings and dates in mixed formats
- RunSettings: one frozen dataclass for the columns, calendar, period-end
  windows, thresholds and word lists, passed to run_python_tests,
  tests_not_run, the IDEA stand-in and write_working_paper, which states it
  on the cover. Replaces their separate keyword arguments (breaking).
- Settings now reach the tests: custom manual_values and the seldom
  threshold went on the cover but not into the tests.
- rules.parse_dates: ISO dates first, then the inferred format, then the rest
  one by one, ambiguous dates day first by default. pandas alone blanked
  every date in a second format.
- Benchmark figures unchanged (re-run reproduces 0.4.0 exactly).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample_priority_list.xlsx
+++ b/docs/sample_priority_list.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -528,159 +528,163 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Parameter: Weekend days</t>
+          <t>Parameter: Period-end windows</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Saturday, Sunday</t>
+          <t>last 3 and first 2 days of each quarter; 5 working days either side of the year-end</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Parameter: Public holidays</t>
+          <t>Parameter: Weekend days</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AE calendar (holidays package 0.106)</t>
+          <t>Saturday, Sunday</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Parameter: Manual entries</t>
+          <t>Parameter: Public holidays</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Source is Manual (case ignored)</t>
+          <t>AE calendar (holidays package 0.106)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Parameter: Seldom-used account</t>
+          <t>Parameter: Dates</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3 entries or fewer</t>
+          <t>ambiguous dates read day first (02/03 is 2 March)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parameter: Keywords</t>
+          <t>Parameter: Manual entries</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>adjust, write off, reversal, correction, director, related party, cash advance, settlement, no invoice, suspense</t>
+          <t>Source is Manual (case ignored)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Parameter: Generic narration words</t>
+          <t>Parameter: Weekend, holiday and round-amount tests</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>adj, adjustment, adjusting, jv, je, journal, entry, correction, reclass, misc, miscellaneous, other, general, various, sundry, test, tbd, being</t>
+          <t>manual lines only</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Parameter: Large amount</t>
+          <t>Parameter: Round amount</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 times the median non-zero amount, used in "why selected" only when performance materiality isn't set (practical judgement)</t>
+          <t>multiple of 10,000</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Parameter: Period-end windows</t>
+          <t>Parameter: Seldom-used account</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>last 3 and first 2 days of each quarter; 5 working days either side of the year-end</t>
+          <t>3 entries or fewer</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Parameter: Weekend, holiday and round-amount tests</t>
+          <t>Parameter: Keywords</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>manual lines only</t>
+          <t>adjust, write off, reversal, correction, director, related party, cash advance, settlement, no invoice, suspense</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Parameter: Round amount</t>
+          <t>Parameter: Generic narration words</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>multiple of 10,000</t>
+          <t>adj, adjustment, adjusting, jv, je, journal, entry, correction, reclass, misc, miscellaneous, other, general, various, sundry, test, tbd, being</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parameter: List size</t>
+          <t>Parameter: Large amount</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0.577 x square root of the ledger lines, within 20-150</t>
+          <t>10 times the median non-zero amount, used in "why selected" only when performance materiality isn't set (practical judgement)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Date run (UTC)</t>
+          <t>Parameter: List size</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>0.577 x square root of the ledger lines, within 20-150</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Prepared by</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
+          <t>Date run (UTC)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Reviewed by</t>
+          <t>Prepared by</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -688,10 +692,18 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Reviewed by</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>See the Method sheet. Internal to the audit team: not for the client.</t>
         </is>

</xml_diff>

<commit_message>
v0.5.1: dates that stopped the pipeline; every column in RunSettings
- parse_dates: one date type for every pass (microsecond times, ISO
  offsets and numbers raised errors); offsets dropped keeping local time;
  numbers 20,000-80,000 read as Excel serial dates.
- Isolation Forest features use parse_dates and RunSettings.
- RunSettings gains account_col, creator_col, approver_col and
  duplicate_key (breaking); the duplicate key is defined once and stated
  on the cover.
- Seldom threshold wording for real IDEA exports (SELDOM_MAX).
- Benchmark figures unchanged (re-run byte-identical to 0.5.0).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample_priority_list.xlsx
+++ b/docs/sample_priority_list.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ambiguous dates read day first (02/03 is 2 March)</t>
+          <t>ambiguous dates read day first (02/03 is 2 March); numbers from 20,000 to 80,000 read as Excel serial dates; time-zone offsets dropped, local time kept</t>
         </is>
       </c>
     </row>
@@ -617,82 +617,86 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3 entries or fewer</t>
+          <t>3 entries or fewer (with real IDEA exports, the threshold the macro was run with: keep it in step with SELDOM_MAX)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Parameter: Keywords</t>
+          <t>Parameter: Duplicate key</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>adjust, write off, reversal, correction, director, related party, cash advance, settlement, no invoice, suspense</t>
+          <t>Date, Account, Description and the amount</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Parameter: Generic narration words</t>
+          <t>Parameter: Keywords</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>adj, adjustment, adjusting, jv, je, journal, entry, correction, reclass, misc, miscellaneous, other, general, various, sundry, test, tbd, being</t>
+          <t>adjust, write off, reversal, correction, director, related party, cash advance, settlement, no invoice, suspense</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parameter: Large amount</t>
+          <t>Parameter: Generic narration words</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10 times the median non-zero amount, used in "why selected" only when performance materiality isn't set (practical judgement)</t>
+          <t>adj, adjustment, adjusting, jv, je, journal, entry, correction, reclass, misc, miscellaneous, other, general, various, sundry, test, tbd, being</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Parameter: List size</t>
+          <t>Parameter: Large amount</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0.577 x square root of the ledger lines, within 20-150</t>
+          <t>10 times the median non-zero amount, used in "why selected" only when performance materiality isn't set (practical judgement)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Date run (UTC)</t>
+          <t>Parameter: List size</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>0.577 x square root of the ledger lines, within 20-150</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Prepared by</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
+          <t>Date run (UTC)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Reviewed by</t>
+          <t>Prepared by</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -700,10 +704,18 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Reviewed by</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>See the Method sheet. Internal to the audit team: not for the client.</t>
         </is>

</xml_diff>